<commit_message>
Working dispatcher, needs some fine tuning
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ChaitanyaRavindra\Documents\UiPath\Dispatcher-ConocoPhillips\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D10100F5-A077-4248-B469-67C4BEB2DA68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{440E431D-4D3C-4CE5-8CAB-660552A23585}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{90EB293F-55A6-4E77-8D34-81D8A5FD87C6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{90EB293F-55A6-4E77-8D34-81D8A5FD87C6}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
     <sheet name="Constants" sheetId="2" r:id="rId2"/>
+    <sheet name="Assets" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="58">
   <si>
     <t>Name</t>
   </si>
@@ -54,9 +55,6 @@
     <t>OrchestratorQueueName</t>
   </si>
   <si>
-    <t>InvoicePath</t>
-  </si>
-  <si>
     <t>Orchestrator queue Name. The value must match with the queue name defined on Orchestrator.</t>
   </si>
   <si>
@@ -91,19 +89,151 @@
   </si>
   <si>
     <t>Data\Input</t>
+  </si>
+  <si>
+    <t>SettlementStatements</t>
+  </si>
+  <si>
+    <t>log1</t>
+  </si>
+  <si>
+    <t>log2</t>
+  </si>
+  <si>
+    <t>log3</t>
+  </si>
+  <si>
+    <t>log4</t>
+  </si>
+  <si>
+    <t>log5</t>
+  </si>
+  <si>
+    <t>log6</t>
+  </si>
+  <si>
+    <t>log7</t>
+  </si>
+  <si>
+    <t>MaxRetryNumber</t>
+  </si>
+  <si>
+    <t>Must be 0 if working with Orchestrator queues. If &gt; 0, the robot will retry the same transaction which failed with a system exception. Must be an integer value.</t>
+  </si>
+  <si>
+    <t>MaxConsecutiveSystemExceptions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The number of consecutive system exceptions allowed. If MaxConsecutiveSystemExceptions is reached, the job is stopped. To disable this feature, set the value to 0. </t>
+  </si>
+  <si>
+    <t>ExScreenshotsFolderPath</t>
+  </si>
+  <si>
+    <t>Exceptions_Screenshots</t>
+  </si>
+  <si>
+    <t>Where to save exceptions screenshots - can be a full or a relative path.</t>
+  </si>
+  <si>
+    <t>LogMessage_GetTransactionData</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Processing Transaction Number: </t>
+  </si>
+  <si>
+    <t>Static part of logging message. Calling Get Transaction Data.</t>
+  </si>
+  <si>
+    <t>LogMessage_GetTransactionDataError</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Error getting transaction data for Transaction Number: </t>
+  </si>
+  <si>
+    <t>Static part of logging message. Error retrieving Transaction Data.</t>
+  </si>
+  <si>
+    <t>LogMessage_Success</t>
+  </si>
+  <si>
+    <t>Transaction Successful.</t>
+  </si>
+  <si>
+    <t>Static part of logging message. Processed Transaction succesful.</t>
+  </si>
+  <si>
+    <t>LogMessage_BusinessRuleException</t>
+  </si>
+  <si>
+    <t>Business rule exception.</t>
+  </si>
+  <si>
+    <t>Static part of logging message. Processed Transaction failed with business exception.</t>
+  </si>
+  <si>
+    <t>LogMessage_ApplicationException</t>
+  </si>
+  <si>
+    <t>System exception.</t>
+  </si>
+  <si>
+    <t>Static part of logging message. Processed Transaction failed with application exception.</t>
+  </si>
+  <si>
+    <t>ExceptionMessage_ConsecutiveErrors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The maximum number of consecutive system exceptions was reached. </t>
+  </si>
+  <si>
+    <t>Error message in case MaxConsecutiveSystemExceptions number is reached.</t>
+  </si>
+  <si>
+    <t>RetryNumberGetTransactionItem</t>
+  </si>
+  <si>
+    <t>The number of times Get Transaction Item activity is retried in case of an exception. Must be an integer &gt;= 1.</t>
+  </si>
+  <si>
+    <t>RetryNumberSetTransactionStatus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The number of times Set transaction status activity is retried in case of an exception. Must be an integer &gt;= 1. </t>
+  </si>
+  <si>
+    <t>ShouldMarkJobAsFaulted</t>
+  </si>
+  <si>
+    <t>Must be TRUE or FALSE. If the value is TRUE and an error occurs in Initialization state or the MaxConsecutiveSystemExceptions is reached, the job is marked as Faulted.</t>
+  </si>
+  <si>
+    <t>Asset</t>
+  </si>
+  <si>
+    <t>OrchestratorAssetFolder</t>
+  </si>
+  <si>
+    <t>Description (Assets will always overwrite other config)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF464E55"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -126,8 +256,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -462,7 +593,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70FDF715-633A-48E2-94DC-A47720AADFAC}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
@@ -485,56 +616,250 @@
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
         <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
         <v>9</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>10</v>
-      </c>
-      <c r="C5" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF1EE7F7-C9B3-42C4-8373-94678C07E5B0}">
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="64.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="150.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>49</v>
+      </c>
+      <c r="B14">
+        <v>2</v>
+      </c>
+      <c r="C14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15">
+        <v>2</v>
+      </c>
+      <c r="C15" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" t="b">
+        <v>0</v>
+      </c>
+      <c r="C17" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -542,11 +867,32 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF1EE7F7-C9B3-42C4-8373-94678C07E5B0}">
-  <dimension ref="A1"/>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7ACA9B3-2CB7-4592-A428-09808A944227}">
+  <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="49.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>